<commit_message>
Add comprehensive debug logging to database operations for deployment troubleshooting
</commit_message>
<xml_diff>
--- a/event_category/events.xlsx
+++ b/event_category/events.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -475,6 +475,316 @@
       <c r="L1" t="inlineStr">
         <is>
           <t>Event URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Helgäventyr i Tensta</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Tensta</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Tensta</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>all_ages</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Lek, matte och kreativitet väntar hos Tekniska filial i Tensta. Fredag till söndag öppnar Tekniska i Tensta dörrarna för dig som är nyfiken, kreativ och vill upptäcka matte på ett helt nytt sätt. Bygg robotar, skapa musik, testa AI och lös kluriga kodgåtor – helt utan krav, bara lust och nyfikenhet.</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>https://www.tekniskamuseet.se/pa-gang/helgaventyr-i-tensta/?date=</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Connect to Learn 2: Elektronik och programmering</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Tensta</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>12-15, Tensta</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>teens</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Vill du ta dina programmeringskunskaper till nästa nivå och förstå hur elektronik fungerar i praktiken? Välkommen till Connect to Learn 2! En klubb för dig mellan 12 och 15 år som vill lära dig MicroPython, elektronik och programmeringslogik på riktigt. Här i Tekniska museets filial i Tensta får du utforska hur kod blir till praktiska lösningar i vardagen.</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>https://www.tekniskamuseet.se/pa-gang/connect-to-learn-elektronik-och-programmering/?date=</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Föräldralediga fredagar på Tekniska</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Tekniska museet</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>0-6</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>preschool</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Här hittar du en självservering på leksaker, nya intryck och skoj. Sinneslabbet är en rolig, trygg och lärorik miljö för barn utan och med funktionsvariationer. Det är framtaget för att stimulera nyfikenhet, lust och lärande. Genom lek och socialt samspel kan de i lugn och ro utveckla sin förmåga att utforska; testa, känna, lukta, se och lära med hjälp av alla sina sinnen. Sinneslabbet är öppet kl10.00 – 13.00på föräldralediga fredagar.</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>https://www.tekniskamuseet.se/pa-gang/foraldralediga-fredagar-pa-tekniska/?date=</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Demostage med Stockholms universitet – Testa framtidens spel</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Tekniska museet</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>all_ages</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Magic of NimurathEtt turbaserat, taktiskt roguelike där spelaren bygger och leder ett party på rutbaserade slagfält, förstärkt av ett kortlekssystem som påverkar strider. Framgång bygger på långsiktiga beslut, smart användning av kort och hur partyt utvecklas under spelets gång.Utvecklat av:Carl-Henrik Huusko, Vincent Blossborn, Carl Roos, Malte Gundhus, Carl-Johan Larson Eliasson, Joel Larsson Wendt, Alexander Olsson, Joel Widemåne, Leo Ferrarini, Hugo Lindgren och Samuel Lövenklev.</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>https://www.tekniskamuseet.se/pa-gang/testa-framtidens-spel-stockholm-universitet/?date=</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Klubb: Upptäck matematik</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Tensta</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>10-12, Tensta</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>teens</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>I den här klubben får du utforska matematik på ett kreativt och lekfullt sätt – genom spel, logik och programmering! Vi analyserar klassiska spel, testar strategier, löser kluriga problem och bygger förståelse för sannolikhet, risk och mönster. Du får prova på robotik, räkna möjliga utfall i spel och upptäcka hur matte kan användas för att fatta smarta beslut.</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>https://www.tekniskamuseet.se/pa-gang/klubb-upptack-matematik/?date=</t>
         </is>
       </c>
     </row>

</xml_diff>